<commit_message>
Reworked Thoughtweave Serum and made parries instakill phantoms and vexes
</commit_message>
<xml_diff>
--- a/src/main/resources/Music Tracks.xlsx
+++ b/src/main/resources/Music Tracks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\etsta\Documents\Minecraft Mods\dndreams-ascend\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\etsta\Documents\Modding MC\dndreams\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C76F7E9-6CA9-4226-9E39-4686577B46AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{985F07A5-E344-488C-A146-EABBABE345A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="76">
   <si>
     <t>Track</t>
   </si>
@@ -51,9 +51,6 @@
     <t>Elrunez</t>
   </si>
   <si>
-    <t>Moderate Motifs</t>
-  </si>
-  <si>
     <t>Ender Dragon #1</t>
   </si>
   <si>
@@ -186,9 +183,6 @@
     <t>Fallen Sentinel</t>
   </si>
   <si>
-    <t>Major</t>
-  </si>
-  <si>
     <t>Dreams of the Future</t>
   </si>
   <si>
@@ -198,29 +192,74 @@
     <t>Plays as the player approaches the sleeping Ender Dragon.</t>
   </si>
   <si>
+    <t>Elrunez, Affliction, Madness</t>
+  </si>
+  <si>
+    <t>Major -&gt; Minor</t>
+  </si>
+  <si>
+    <t>Demons of the Past</t>
+  </si>
+  <si>
+    <t>Elrunez, Death</t>
+  </si>
+  <si>
+    <t>Elrunez, Madness, Death</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Minor?</t>
+  </si>
+  <si>
+    <t>Minor/Major</t>
+  </si>
+  <si>
+    <t>Madness, Affliction</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>The Weight of Your Demons</t>
+  </si>
+  <si>
+    <t>The Weight of Your Dreams</t>
+  </si>
+  <si>
+    <t>No Survivors</t>
+  </si>
+  <si>
+    <t>Against the Guiding Light</t>
+  </si>
+  <si>
+    <t>Fateful Approach</t>
+  </si>
+  <si>
+    <t>A Home that Isn't</t>
+  </si>
+  <si>
+    <t>The Nightmare Storm</t>
+  </si>
+  <si>
+    <t>The nightmare storms plague the Spirit World, appearing just as quickly as they vanish. They are accompanied by an influx of hostile creatures.</t>
+  </si>
+  <si>
     <t>Madness</t>
   </si>
   <si>
-    <t>Elrunez, Affliction, Madness</t>
-  </si>
-  <si>
-    <t>Major -&gt; Minor</t>
-  </si>
-  <si>
-    <t>Demons of the Past</t>
-  </si>
-  <si>
-    <t>Elrunez, Death</t>
-  </si>
-  <si>
-    <t>Elrunez, Madness, Death</t>
+    <t>Mental Mire</t>
+  </si>
+  <si>
+    <t>Dance the Spears of Judgment</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -237,6 +276,15 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <i/>
       <sz val="11"/>
       <color theme="1"/>
@@ -299,7 +347,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -323,6 +371,9 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Heading 1" xfId="1" builtinId="16"/>
@@ -330,6 +381,10 @@
   </cellStyles>
   <dxfs count="8">
     <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -371,15 +426,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{99D8C478-FF24-485C-A27D-740352D838C9}" name="Table3" displayName="Table3" ref="A1:F21" totalsRowShown="0" dataDxfId="6" headerRowBorderDxfId="7" headerRowCellStyle="Heading 1">
-  <autoFilter ref="A1:F21" xr:uid="{99D8C478-FF24-485C-A27D-740352D838C9}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{99D8C478-FF24-485C-A27D-740352D838C9}" name="Table3" displayName="Table3" ref="A1:F22" totalsRowShown="0" dataDxfId="6" headerRowBorderDxfId="7" headerRowCellStyle="Heading 1">
+  <autoFilter ref="A1:F22" xr:uid="{99D8C478-FF24-485C-A27D-740352D838C9}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{44F286B8-39E0-4372-9A35-DD9C96243317}" name="Track" dataDxfId="5"/>
     <tableColumn id="2" xr3:uid="{16734576-B6DD-4BED-933E-7FCEC034B1F2}" name="Description" dataDxfId="4"/>
     <tableColumn id="3" xr3:uid="{BA1F16DB-2CC9-44EF-94CB-EB1AB6A67C09}" name="Important Motifs" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{E9EA6A4B-2A33-4EFE-8731-2A46DBE068DB}" name="Moderate Motifs" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{0FFEA9D9-CF62-4F9D-BB65-1EF2F32FF522}" name="Acknowledged Motifs" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{F324D180-2C48-490B-8FC2-ADD1A2924471}" name="Key" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{0FFEA9D9-CF62-4F9D-BB65-1EF2F32FF522}" name="Acknowledged Motifs" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{F324D180-2C48-490B-8FC2-ADD1A2924471}" name="Key" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{6935513B-A5AD-4EAD-9AE2-DB9E806C56C2}" name="Name" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleDark11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -648,19 +703,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G22"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.28515625" customWidth="1"/>
-    <col min="2" max="2" width="63.28515625" customWidth="1"/>
-    <col min="3" max="3" width="21.28515625" customWidth="1"/>
-    <col min="4" max="4" width="23.85546875" customWidth="1"/>
-    <col min="5" max="5" width="28.28515625" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" customWidth="1"/>
-    <col min="8" max="8" width="23.42578125" customWidth="1"/>
+    <col min="1" max="1" width="18.33203125" customWidth="1"/>
+    <col min="2" max="2" width="63.33203125" customWidth="1"/>
+    <col min="3" max="3" width="21.33203125" customWidth="1"/>
+    <col min="4" max="4" width="23.88671875" customWidth="1"/>
+    <col min="5" max="5" width="13.109375" customWidth="1"/>
+    <col min="6" max="6" width="33.21875" customWidth="1"/>
+    <col min="7" max="7" width="20.109375" customWidth="1"/>
+    <col min="8" max="8" width="23.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="20.399999999999999" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -668,19 +724,19 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="E1" s="3" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="30.75" thickTop="1" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="29.4" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>2</v>
       </c>
@@ -690,337 +746,379 @@
       <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="2"/>
+      <c r="D2" s="2" t="s">
+        <v>5</v>
+      </c>
       <c r="E2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+      <c r="F2" s="11"/>
+    </row>
+    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F3" s="11"/>
+      <c r="G3" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>5</v>
       </c>
       <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="E4" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="F4" s="11"/>
+      <c r="G4" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>5</v>
       </c>
       <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="E5" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F5" s="11"/>
+    </row>
+    <row r="6" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C6" s="2"/>
       <c r="D6" s="2" t="s">
-        <v>41</v>
+        <v>7</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+      <c r="F6" s="11"/>
+    </row>
+    <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="E7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="72" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="45" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="2"/>
+      <c r="C9" s="2" t="s">
+        <v>59</v>
+      </c>
       <c r="D9" s="2" t="s">
-        <v>62</v>
+        <v>17</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F9" s="2"/>
-    </row>
-    <row r="10" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="2"/>
+      <c r="D10" s="2" t="s">
+        <v>20</v>
+      </c>
       <c r="E10" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A12" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="45" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="60" x14ac:dyDescent="0.25">
-      <c r="A13" s="9" t="s">
-        <v>52</v>
+      <c r="D12" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="F12" s="11"/>
+    </row>
+    <row r="13" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A13" s="8" t="s">
+        <v>21</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>5</v>
       </c>
       <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-    </row>
-    <row r="14" spans="1:8" ht="60" x14ac:dyDescent="0.25">
-      <c r="A14" s="8" t="s">
-        <v>29</v>
+      <c r="E13" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F13" s="11"/>
+    </row>
+    <row r="14" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A14" s="9" t="s">
+        <v>51</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F14" s="11"/>
+    </row>
+    <row r="15" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F14" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
+      <c r="E15" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C16" s="2" t="s">
+      <c r="C17" s="2" t="s">
         <v>4</v>
-      </c>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="60" x14ac:dyDescent="0.25">
-      <c r="A17" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>7</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F17" s="11"/>
+    </row>
+    <row r="18" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A19" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F20" s="11"/>
+    </row>
+    <row r="21" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A21" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F21" s="11" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A22" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F17" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A19" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F19" s="2"/>
-    </row>
-    <row r="20" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-    </row>
-    <row r="21" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A21" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E21" s="2" t="s">
+      <c r="D22" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F21" s="2" t="s">
-        <v>59</v>
-      </c>
+      <c r="E22" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="F22" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
New Version of Mindburn 🔥
</commit_message>
<xml_diff>
--- a/src/main/resources/Music Tracks.xlsx
+++ b/src/main/resources/Music Tracks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\etsta\Documents\Modding MC\dndreams\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{985F07A5-E344-488C-A146-EABBABE345A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DACE305-C106-4026-A32A-F7BB60196260}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="78">
   <si>
     <t>Track</t>
   </si>
@@ -198,9 +198,6 @@
     <t>Major -&gt; Minor</t>
   </si>
   <si>
-    <t>Demons of the Past</t>
-  </si>
-  <si>
     <t>Elrunez, Death</t>
   </si>
   <si>
@@ -253,13 +250,47 @@
   </si>
   <si>
     <t>Dance the Spears of Judgment</t>
+  </si>
+  <si>
+    <t>Mindburn</t>
+  </si>
+  <si>
+    <t>Demons from the Past</t>
+  </si>
+  <si>
+    <r>
+      <t>Cold, Calculated Wrath</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> +</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Burning, Scornful Pride</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -286,6 +317,14 @@
     <font>
       <b/>
       <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -733,7 +772,7 @@
         <v>49</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="29.4" thickTop="1" x14ac:dyDescent="0.3">
@@ -762,17 +801,19 @@
         <v>48</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>7</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="F3" s="11"/>
+        <v>59</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>75</v>
+      </c>
       <c r="G3" s="4" t="s">
-        <v>57</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -787,7 +828,7 @@
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F4" s="11"/>
       <c r="G4" s="5" t="s">
@@ -806,7 +847,7 @@
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F5" s="11"/>
     </row>
@@ -843,7 +884,7 @@
         <v>50</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -854,14 +895,14 @@
         <v>10</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -872,7 +913,7 @@
         <v>11</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>17</v>
@@ -881,7 +922,7 @@
         <v>50</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -901,25 +942,25 @@
         <v>50</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>73</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -936,9 +977,11 @@
         <v>4</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="F12" s="11"/>
+        <v>60</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="13" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
@@ -986,10 +1029,10 @@
         <v>7</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -1004,10 +1047,10 @@
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -1043,7 +1086,7 @@
         <v>50</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -1060,10 +1103,10 @@
         <v>20</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -1080,7 +1123,7 @@
         <v>20</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F20" s="11"/>
     </row>
@@ -1096,10 +1139,10 @@
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Not sure when I did this, but sure
</commit_message>
<xml_diff>
--- a/src/main/resources/Music Tracks.xlsx
+++ b/src/main/resources/Music Tracks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\etsta\Documents\Modding MC\dndreams\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DACE305-C106-4026-A32A-F7BB60196260}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A607A44D-143D-4AC4-A1D5-52731F452952}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="79">
   <si>
     <t>Track</t>
   </si>
@@ -284,6 +284,9 @@
       </rPr>
       <t xml:space="preserve"> Burning, Scornful Pride</t>
     </r>
+  </si>
+  <si>
+    <t>Tales from Otherwhere</t>
   </si>
 </sst>
 </file>
@@ -332,7 +335,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -363,6 +366,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -386,7 +395,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -413,6 +422,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Heading 1" xfId="1" builtinId="16"/>
@@ -850,6 +860,9 @@
         <v>59</v>
       </c>
       <c r="F5" s="11"/>
+      <c r="G5" s="12" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="6" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
@@ -946,7 +959,7 @@
       </c>
     </row>
     <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="7" t="s">
         <v>70</v>
       </c>
       <c r="B11" s="2" t="s">
@@ -964,7 +977,7 @@
       </c>
     </row>
     <row r="12" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="8" t="s">
         <v>30</v>
       </c>
       <c r="B12" s="2" t="s">
@@ -984,7 +997,7 @@
       </c>
     </row>
     <row r="13" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="9" t="s">
         <v>21</v>
       </c>
       <c r="B13" s="2" t="s">
@@ -1000,7 +1013,7 @@
       <c r="F13" s="11"/>
     </row>
     <row r="14" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="8" t="s">
         <v>51</v>
       </c>
       <c r="B14" s="2" t="s">
@@ -1016,7 +1029,7 @@
       <c r="F14" s="11"/>
     </row>
     <row r="15" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="8" t="s">
+      <c r="A15" s="9" t="s">
         <v>28</v>
       </c>
       <c r="B15" s="2" t="s">
@@ -1036,7 +1049,7 @@
       </c>
     </row>
     <row r="16" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="9" t="s">
+      <c r="A16" s="8" t="s">
         <v>27</v>
       </c>
       <c r="B16" s="2" t="s">
@@ -1054,7 +1067,7 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="9" t="s">
         <v>24</v>
       </c>
       <c r="B17" s="2" t="s">
@@ -1070,7 +1083,7 @@
       <c r="F17" s="11"/>
     </row>
     <row r="18" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="9" t="s">
+      <c r="A18" s="8" t="s">
         <v>18</v>
       </c>
       <c r="B18" s="2" t="s">
@@ -1090,7 +1103,7 @@
       </c>
     </row>
     <row r="19" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="9" t="s">
         <v>46</v>
       </c>
       <c r="B19" s="2" t="s">
@@ -1110,7 +1123,7 @@
       </c>
     </row>
     <row r="20" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A20" s="9" t="s">
+      <c r="A20" s="8" t="s">
         <v>44</v>
       </c>
       <c r="B20" s="2" t="s">
@@ -1128,7 +1141,7 @@
       <c r="F20" s="11"/>
     </row>
     <row r="21" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A21" s="8" t="s">
+      <c r="A21" s="9" t="s">
         <v>32</v>
       </c>
       <c r="B21" s="2" t="s">
@@ -1146,7 +1159,7 @@
       </c>
     </row>
     <row r="22" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A22" s="9" t="s">
+      <c r="A22" s="8" t="s">
         <v>34</v>
       </c>
       <c r="B22" s="2" t="s">

</xml_diff>